<commit_message>
Phase 10: Separate incineration LCA from landfill LCA
- Provider IS_Rejected: GWPActualProcess now uses 3-stage combustion GWP
  factors (drying + thermalDecomp + slagFormation) instead of GWPWasteToLandfill
- Intermediate: new variables gwpFactor_drying/thermalDecomp/slagFormation
  read from Intermediate sheet B15-17 at startup
- CombustionSink.onEnter: adds per-stage GWP to GWPActualIncineration
  (facility-level reporting, separate from Provider.GWPActualProcess)
- recyclingProcessing(): process waste LCA deferred to pwSink DES
  (pw_pendingGWP/HTP/LUP/CED staged before inject, applied at Sink)
- pwSink.onEnter: applies staged LCA → GWPActualProcess + GWPActualTotal
- Excel Intermediate B15-B17: placeholder combustion GWP factors
  (0.05 / 0.80 / 0.02 kg CO2-eq/kg; ILLUSTRATIVE — update from ecoinvent)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/31MARZ.xlsx
+++ b/31MARZ.xlsx
@@ -480,7 +480,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="75">
+  <cellXfs count="76">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -677,6 +677,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="19" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -9893,8 +9896,8 @@
     <mergeCell ref="A3:A5"/>
     <mergeCell ref="A9:A11"/>
     <mergeCell ref="A15:A17"/>
+    <mergeCell ref="A1:B1"/>
     <mergeCell ref="B3:B5"/>
-    <mergeCell ref="A1:B1"/>
     <mergeCell ref="A6:A8"/>
     <mergeCell ref="A18:A20"/>
   </mergeCells>
@@ -10306,7 +10309,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.25" customHeight="1"/>
   <cols>
     <col width="28" customWidth="1" style="67" min="1" max="1"/>
@@ -10670,6 +10673,81 @@
       <c r="F14" s="70" t="inlineStr">
         <is>
           <t>⚠ TODO BEFORE FINAL RESULTS (2026-03-31): This emission factor is taken from the general literature (see Source/Rationale, col E). It has NOT been verified against VSIP1-specific or BIWASE-specific waste composition data. Before submitting thesis results, replace with: (1) measured calorific value and elemental analysis of the actual waste stream at BIWASE, (2) BIWASE/ESCAR operational emission monitoring data if available (ADB 56118-001), (3) or validated ecoinvent 3.9 process for the actual material mix. Current value is ILLUSTRATIVE ONLY.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>gwpFactor_drying_kgCO2eqPerKg</t>
+        </is>
+      </c>
+      <c r="B15" s="75" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>kg CO2-eq / kg waste</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>GWP emission factor for waste drying stage in batch incineration. Represents GHG from moisture evaporation and pre-heating (indirect energy and steam release). ILLUSTRATIVE — replace with ecoinvent 3.9 process data before thesis submission.</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>IPCC 2006 NGGIP Vol.5 Ch.5; Arena 2012 (Waste Management). Placeholder 0.05 kg CO2-eq/kg. Lower bound of drying-stage GHG: typically 2–8% of total incineration impact.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>gwpFactor_thermalDecomp_kgCO2eqPerKg</t>
+        </is>
+      </c>
+      <c r="B16" s="75" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>kg CO2-eq / kg waste</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>GWP emission factor for thermal decomposition stage (primary combustion chamber, 850–1000°C). Represents direct CO2 from oxidation of organic fraction. ILLUSTRATIVE — replace with ecoinvent 3.9 process data.</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>IPCC 2006 mixed waste combustion EF: 0.8–1.1 kg CO2/kg (wet basis). Value 0.80 used here (lower end for mixed industrial waste with significant inorganic fraction). Update with BIWASE-specific fuel characterisation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>gwpFactor_slagFormation_kgCO2eqPerKg</t>
+        </is>
+      </c>
+      <c r="B17" s="75" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>kg CO2-eq / kg waste</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>GWP emission factor for slag/ash formation stage (bottom ash stabilisation and residue handling). Represents residual oxidation and mineral carbonation reactions producing bottom ash. ILLUSTRATIVE — replace with ecoinvent data.</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Estimated from ecoinvent 3.9 "treatment of municipal solid waste, incineration" process. Slag-related GHG typically &lt;5% of total incineration GWP. 0.02 kg CO2-eq/kg used as indicative value.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Excel: add ecoinvent 3.9 comments to B15-17, verification flags, todo row
- Cell comments on Intermediate!B15-17: ecoinvent query 'treatment of
  municipal solid waste by incineration' (RoW), replacement guidance
- F15-17 Verification Flag column populated with NOT VERIFIED notice
- 'to do before submitting' row 9: High-priority task to replace
  illustrative GWP stage factors with validated ecoinvent 3.9 data

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/31MARZ.xlsx
+++ b/31MARZ.xlsx
@@ -758,6 +758,52 @@
 </styleSheet>
 </file>
 
+<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>CE3.0 Model</author>
+  </authors>
+  <commentList>
+    <comment ref="B15" authorId="0" shapeId="0">
+      <text>
+        <t>⚠ ECOINVENT REPLACEMENT REQUIRED
+Current value 0.05 is ILLUSTRATIVE.
+Recommended ecoinvent 3.9 query:
+  'treatment of municipal solid waste by incineration'
+  → select 'drying / pre-treatment' subprocess if available,
+    or allocate ~3–8% of total incineration GWP to this stage.
+For SE Asian context: use ecoinvent RoW (rest-of-world) process.
+Replace before thesis submission.</t>
+      </text>
+    </comment>
+    <comment ref="B16" authorId="0" shapeId="0">
+      <text>
+        <t>⚠ ECOINVENT REPLACEMENT REQUIRED
+Current value 0.80 is ILLUSTRATIVE (IPCC 2006 range: 0.8–1.1).
+Recommended ecoinvent 3.9 query:
+  'treatment of municipal solid waste by incineration'
+  → use total incineration GWP factor for thermal decomp stage,
+    or adopt the full process GWP as a single conservative factor.
+For SE Asian context: use ecoinvent RoW (rest-of-world) process.
+Replace before thesis submission.</t>
+      </text>
+    </comment>
+    <comment ref="B17" authorId="0" shapeId="0">
+      <text>
+        <t>⚠ ECOINVENT REPLACEMENT REQUIRED
+Current value 0.02 is ILLUSTRATIVE.
+Recommended ecoinvent 3.9 query:
+  'treatment of municipal solid waste by incineration'
+  → slag/bottom ash sub-process or residue handling GWP.
+Typically &lt;5% of total incineration GWP.
+For SE Asian context: use ecoinvent RoW (rest-of-world) process.
+Replace before thesis submission.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -9896,8 +9942,8 @@
     <mergeCell ref="A3:A5"/>
     <mergeCell ref="A9:A11"/>
     <mergeCell ref="A15:A17"/>
+    <mergeCell ref="B3:B5"/>
     <mergeCell ref="A1:B1"/>
-    <mergeCell ref="B3:B5"/>
     <mergeCell ref="A6:A8"/>
     <mergeCell ref="A18:A20"/>
   </mergeCells>
@@ -10700,6 +10746,11 @@
           <t>IPCC 2006 NGGIP Vol.5 Ch.5; Arena 2012 (Waste Management). Placeholder 0.05 kg CO2-eq/kg. Lower bound of drying-stage GHG: typically 2–8% of total incineration impact.</t>
         </is>
       </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>⚠ NOT VERIFIED — replace with ecoinvent 3.9 'treatment of municipal solid waste by incineration' (RoW) before thesis submission</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -10725,6 +10776,11 @@
           <t>IPCC 2006 mixed waste combustion EF: 0.8–1.1 kg CO2/kg (wet basis). Value 0.80 used here (lower end for mixed industrial waste with significant inorganic fraction). Update with BIWASE-specific fuel characterisation.</t>
         </is>
       </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>⚠ NOT VERIFIED — replace with ecoinvent 3.9 'treatment of municipal solid waste by incineration' (RoW) before thesis submission</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -10748,6 +10804,11 @@
       <c r="E17" t="inlineStr">
         <is>
           <t>Estimated from ecoinvent 3.9 "treatment of municipal solid waste, incineration" process. Slag-related GHG typically &lt;5% of total incineration GWP. 0.02 kg CO2-eq/kg used as indicative value.</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>⚠ NOT VERIFIED — replace with ecoinvent 3.9 'treatment of municipal solid waste by incineration' (RoW) before thesis submission</t>
         </is>
       </c>
     </row>
@@ -10757,6 +10818,7 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="300" verticalDpi="300"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -11026,7 +11088,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.25" customHeight="1"/>
   <cols>
     <col width="14" customWidth="1" style="67" min="1" max="1"/>
@@ -11265,6 +11327,33 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Replace ILLUSTRATIVE combustion GWP stage factors (B15–B17 in Intermediate sheet) with validated ecoinvent 3.9 values. Query: 'treatment of municipal solid waste by incineration' (ecoinvent 3.9, RoW process). Assign GWP proportionally to drying, thermal decomposition, and slag formation stages, or use full-process factor conservatively at thermal stage (B16). Also update source citations in column E of Intermediate sheet.</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Affects GWPActualIncineration (Intermediate) and GWPActualProcess (Provider non-IS path). AnyLogic reads: Intermediate!B15 (drying), B16 (thermalDecomp), B17 (slagFormation). chkRange bounds: 0.0–10.0 kg CO2-eq/kg. Both CombustionSink.onEnter and Provider IS_Rejected state use these factors.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Phase 11: HTP/LUP/CED combustion factors + recycling DES ecoinvent comments
ALP changes:
- 3 new Intermediate variables: htpFactor_incineration_CTUhPerKg (B18),
  lupFactor_incineration_m2yrPerKg (B19), cedFactor_incineration_MJPerKg (B20)
- Main startup: getCellNumericValue + chkRange for B18-B20
- Provider IS_Rejected: HTP/LUP/CED now use combustion-specific factors
  instead of WasteToLandfill factors (methodologically consistent)
- CombustionSink.onEnter: diagnostic traceln for all 4 LCA categories
- Recycling DES (recyclShredding/Washing/Separation/Extrusion): onEnter
  fields populated with ecoinvent 3.9 query reminder comments

Excel changes:
- Intermediate rows 18-20: htpFactor/lupFactor/cedFactor incineration
  with orange cells, ecoinvent comments, verification flags (ILLUSTRATIVE)
- to-do sheet row 10: plastic recycling EF search task (High priority)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/31MARZ.xlsx
+++ b/31MARZ.xlsx
@@ -800,6 +800,36 @@
 Replace before thesis submission.</t>
       </text>
     </comment>
+    <comment ref="B18" authorId="0" shapeId="0">
+      <text>
+        <t>⚠ ECOINVENT REPLACEMENT REQUIRED
+Current value 2.5e-9 CTUh/kg is ILLUSTRATIVE.
+Recommended ecoinvent 3.9 query:
+  'treatment of municipal solid waste by incineration'
+  → select HTP characterisation factor (RoW process).
+Replace before thesis submission.</t>
+      </text>
+    </comment>
+    <comment ref="B19" authorId="0" shapeId="0">
+      <text>
+        <t>⚠ ECOINVENT REPLACEMENT REQUIRED
+Current value 0.002 m2yr/kg is ILLUSTRATIVE.
+Recommended ecoinvent 3.9 query:
+  'treatment of municipal solid waste by incineration'
+  → select LUP characterisation factor (RoW process).
+Replace before thesis submission.</t>
+      </text>
+    </comment>
+    <comment ref="B20" authorId="0" shapeId="0">
+      <text>
+        <t>⚠ ECOINVENT REPLACEMENT REQUIRED
+Current value 0.8 MJ/kg is ILLUSTRATIVE.
+Recommended ecoinvent 3.9 query:
+  'treatment of municipal solid waste by incineration'
+  → select CED (non-renewable) characterisation factor (RoW process).
+Replace before thesis submission.</t>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
@@ -9942,8 +9972,8 @@
     <mergeCell ref="A3:A5"/>
     <mergeCell ref="A9:A11"/>
     <mergeCell ref="A15:A17"/>
+    <mergeCell ref="A1:B1"/>
     <mergeCell ref="B3:B5"/>
-    <mergeCell ref="A1:B1"/>
     <mergeCell ref="A6:A8"/>
     <mergeCell ref="A18:A20"/>
   </mergeCells>
@@ -10355,7 +10385,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:F20"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.25" customHeight="1"/>
   <cols>
     <col width="28" customWidth="1" style="67" min="1" max="1"/>
@@ -10807,6 +10837,96 @@
         </is>
       </c>
       <c r="F17" t="inlineStr">
+        <is>
+          <t>⚠ NOT VERIFIED — replace with ecoinvent 3.9 'treatment of municipal solid waste by incineration' (RoW) before thesis submission</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>htpFactor_incineration_CTUhPerKg</t>
+        </is>
+      </c>
+      <c r="B18" s="68" t="n">
+        <v>2.5e-09</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>CTUh / kg waste</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Human Toxicity Potential (HTP) emission factor for waste incineration at BIWASE. Accounts for toxic emissions (dioxins, heavy metals) from combustion of mixed industrial/MSW waste. ILLUSTRATIVE — replace with ecoinvent 3.9 'treatment of municipal solid waste by incineration' (RoW) before thesis submission.</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Indicative value from ecoinvent 3.9 incineration process characterisation factors (CTUh / kg). Range: 1e-9 to 1e-8 CTUh/kg depending on flue gas treatment level. BIWASE operates bag filter + scrubber — use mid-range estimate. ILLUSTRATIVE ONLY.</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>⚠ NOT VERIFIED — replace with ecoinvent 3.9 'treatment of municipal solid waste by incineration' (RoW) before thesis submission</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>lupFactor_incineration_m2yrPerKg</t>
+        </is>
+      </c>
+      <c r="B19" s="68" t="n">
+        <v>0.002</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>m2yr / kg waste</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Land Use Potential (LUP) emission factor for waste incineration. Represents land occupation for BIWASE facility footprint and ash disposal area per kg processed. ILLUSTRATIVE — replace with ecoinvent 3.9 'treatment of municipal solid waste by incineration' (RoW) before thesis submission.</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Indicative estimate based on ecoinvent 3.9 LUP characterisation for incineration (RoW). LUP is typically small for incineration vs. landfill. ILLUSTRATIVE ONLY.</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>⚠ NOT VERIFIED — replace with ecoinvent 3.9 'treatment of municipal solid waste by incineration' (RoW) before thesis submission</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>cedFactor_incineration_MJPerKg</t>
+        </is>
+      </c>
+      <c r="B20" s="68" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>MJ / kg waste</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Cumulative Energy Demand (CED) for waste incineration at BIWASE. Represents non-renewable primary energy consumed per kg of waste processed (auxiliary fuel, electrical auxiliary loads, flue gas treatment). ILLUSTRATIVE — replace with ecoinvent 3.9 'treatment of municipal solid waste by incineration' (RoW) before thesis submission.</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Indicative value: BIWASE operates a two-chamber incinerator at 850–1000°C with oil/gas auxiliary burner. CED typical range 0.4–1.5 MJ/kg for industrial incineration. ILLUSTRATIVE ONLY — replace with ecoinvent 3.9 RoW process.</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
         <is>
           <t>⚠ NOT VERIFIED — replace with ecoinvent 3.9 'treatment of municipal solid waste by incineration' (RoW) before thesis submission</t>
         </is>
@@ -11088,7 +11208,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.25" customHeight="1"/>
   <cols>
     <col width="14" customWidth="1" style="67" min="1" max="1"/>
@@ -11354,6 +11474,33 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Search and add emission factors for plastic scrap recycling steps (shredding, washing, separation, extrusion) for Vietnam/SE Asia region. ecoinvent 3.9 query: 'treatment of plastic waste, via mechanical recycling' (RoW or CN geography). Add per-step EF rows to Intermediate Excel sheet for all four impact categories: GWP (kg CO2-eq/kg), HTP (CTUh/kg), CED (MJ/kg), LUP (m2yr/kg). Wire into each recyclShredding / recyclWashing / recyclSeparation / recyclExtrusion onEnter action in Intermediate agent. Consider system-expansion credit for avoided virgin polymer at extrusion step — document as explicit methodology choice in thesis.</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Affects GWPActualProcess, HTPActualProcess, LUPActualProcess, CEDActualProcess for the IS pathway. Without these, recycling LCA impact is zero — understates processing cost of the IS route.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Phase 12: Material-specific disposal arrays + 4 new DES chains (thesis refs [63-71])
Changes:
- Main: pw_landfillShare/pw_incinerationShare → double[] arrays (per-material, Consensus-validated)
- Main: noIS_landfillShare[5] / noIS_incinerationShare[5] added for BAU baseline
- Intermediate.recyclingProcessing(): uses pw_landfillSharePerMat[m]/pw_incinerationSharePerMat[m]
- Intermediate.NonIS_Disposal: uses noIS_landfillShare[matIdx] for blended disposal cost
- 4 new DES chains: paper (Bale→Load), FERROUS (Sort→Grade→PreTreat),
  TEXTILE (CutShred→FibreReprocess), NON_FERROUS (Sort→Segregate)
- recyclStart.inject() → per-material conditional inject calls [63-71]
- PLASTIC DES step comments updated to cite thesis ref [63]
- xlsx: Intermediate sheet rows 22-27 updated with array documentation

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/31MARZ.xlsx
+++ b/31MARZ.xlsx
@@ -28,7 +28,7 @@
     <numFmt numFmtId="164" formatCode="#,##0.00000"/>
     <numFmt numFmtId="165" formatCode="_-* #,##0_-;\-* #,##0_-;_-* \-??_-;_-@_-"/>
   </numFmts>
-  <fonts count="30">
+  <fonts count="31">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -206,6 +206,10 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001F497D"/>
     </font>
   </fonts>
   <fills count="20">
@@ -480,7 +484,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="76">
+  <cellXfs count="78">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -681,6 +685,8 @@
     <xf numFmtId="0" fontId="0" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -10385,7 +10391,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F20"/>
+  <dimension ref="A1:F30"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.25" customHeight="1"/>
   <cols>
     <col width="28" customWidth="1" style="67" min="1" max="1"/>
@@ -10932,6 +10938,149 @@
         </is>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" s="76" t="inlineStr">
+        <is>
+          <t>── Process Waste Fate &amp; NoIS Disposal Arrays (Consensus-validated 2026-04-02) ──</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>pw_landfillSharePerMat[]</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>[0.70, 0.80, 0.85, 0.50, 0.85]</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>fraction [PLASTIC/PAPER/Fe/TEXTILE/NFe]</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Hard-coded in ALP Main (not read from Excel). Recycling residue → landfill per material.</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>[LIT] Vietnam ET Journal 2024; SE Asia MSW 2023 (Sustainability); Thai Al LCA 2025 (IOP); Energies 2024 (Textile)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>pw_incinerationSharePerMat[]</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>[0.25, 0.10, 0.05, 0.40, 0.10]</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>fraction [PLASTIC/PAPER/Fe/TEXTILE/NFe]</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Hard-coded in ALP Main (not read from Excel). Recycling residue → incineration per material.</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>[LIT] SE Asia open burning (ES&amp;T 2020); Energies 2024; Thai Al 2025; HCMC MSW 2016</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="76" t="inlineStr">
+        <is>
+          <t>noIS_landfillShare[] / noIS_incinerationShare[]</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>LF:[0.60,0.75,0.15,0.55,0.15] / IN:[0.30,0.10,0.05,0.35,0.05]</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>fraction [PLASTIC/PAPER/Fe/TEXTILE/NFe]</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>BAU disposal (useIS=false). Hard-coded in ALP Main. LF=landfill/open-dump; IN=incineration/open-burning.</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>[LIT] Vietnam TV MFA 2018 (RCR, metals); HCMC MSW 2016; Vietnam plastic 2024; Energies 2024; Thai Al LCA 2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>bottomAsh_massFraction</t>
+        </is>
+      </c>
+      <c r="B26" s="77" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>fraction</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>AnyLogic reads: getCellNumericValue('Intermediate', 26, 2)</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>[LIT] Bottom ash = 25% of incinerated waste mass. IEA Bioenergy Task 36; EU WID reference.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>flyAsh_massFraction</t>
+        </is>
+      </c>
+      <c r="B27" s="77" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>fraction</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>AnyLogic reads: getCellNumericValue('Intermediate', 27, 2)</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>[LIT] Fly ash = 4% mass fraction (hazardous). EU WID 2000/76/EC; ecoinvent 3.9 MSWI reference.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="76" t="n"/>
+    </row>
+    <row r="29"/>
+    <row r="30"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:E1"/>

</xml_diff>

<commit_message>
Phase 13: DES descriptions, disposal array fixes, fleet CAPEX, baseline truck weight
- pwStart/pwTransport/pwLandfillDeposit/pwSink: Description fields added,
  visible in AnyLogic Properties panel when clicking each block
- noIS_landfillShare[0,1] aligned to pw_* for PLASTIC/PAPER: modeling
  assumption subject to sensitivity analysis [ASSUMED]; metals retained
- Fleet CAPEX now wired at t=0: garbageTrucks.size() x truckCapex_SGD
  deducted from npv and intermediate.entityNPV (Phase 3 gap closed)
- truckBaseWeight_t: new param, TruckFleet M3 = 8.0 t [ASSUMED-LIT]
  for deadhead (empty-trip) cost and emission accounting
- Excel: TruckFleet M3 orange, noIS row 25 corrected, HMS1 note row 28
- futurenotes.txt: items [9]-[15] added (grading, non-ferrous, MSW,
  ferrous informal sector, ash fractions, recycling OPEX, sheet consolidation)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/31MARZ.xlsx
+++ b/31MARZ.xlsx
@@ -212,7 +212,7 @@
       <color rgb="001F497D"/>
     </font>
   </fonts>
-  <fills count="20">
+  <fills count="21">
     <fill>
       <patternFill/>
     </fill>
@@ -317,6 +317,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFCC99"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor rgb="FFFFCC99"/>
       </patternFill>
     </fill>
   </fills>
@@ -484,7 +490,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="78">
+  <cellXfs count="79">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -687,6 +693,7 @@
     </xf>
     <xf numFmtId="0" fontId="30" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="19" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="26" fillId="20" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -10235,8 +10242,16 @@
           <t>Source_capacity</t>
         </is>
       </c>
-      <c r="M2" s="61" t="n"/>
-      <c r="N2" s="61" t="n"/>
+      <c r="M2" s="61" t="inlineStr">
+        <is>
+          <t>TruckBaseWeight_t</t>
+        </is>
+      </c>
+      <c r="N2" s="61" t="inlineStr">
+        <is>
+          <t>Source_baseWeight</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="80" customHeight="1" s="67">
       <c r="A3" s="62" t="n">
@@ -10277,8 +10292,14 @@
           <t>WRAP (2022) Baling guidance; EPA (2016) Waste Characterisation Report; Illustrative</t>
         </is>
       </c>
-      <c r="M3" s="61" t="n"/>
-      <c r="N3" s="61" t="n"/>
+      <c r="M3" s="78" t="n">
+        <v>8</v>
+      </c>
+      <c r="N3" s="61" t="inlineStr">
+        <is>
+          <t>Unladen mass ~8 t for medium waste truck (5-10 t payload class). TCVN 7271:2003; [ASSUMED-LIT]</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="27.75" customHeight="1" s="67">
       <c r="A4" s="65" t="n"/>
@@ -10391,7 +10412,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F30"/>
+  <dimension ref="A1:F28"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.25" customHeight="1"/>
   <cols>
     <col width="28" customWidth="1" style="67" min="1" max="1"/>
@@ -11007,7 +11028,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>LF:[0.60,0.75,0.15,0.55,0.15] / IN:[0.30,0.10,0.05,0.35,0.05]</t>
+          <t>LF:[0.70,0.80,0.15,0.55,0.15] / IN:[0.25,0.10,0.05,0.35,0.05]</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -11017,7 +11038,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>BAU disposal (useIS=false). Hard-coded in ALP Main. LF=landfill/open-dump; IN=incineration/open-burning.</t>
+          <t>BAU disposal (useIS=false). Hard-coded in ALP Main. [0],[1] PLASTIC/PAPER aligned to pw_* arrays — modeling assumption subject to sensitivity analysis [ASSUMED]. [2],[4] FERROUS/NON_FERROUS low shares reflect informal scrap dealer diversion (Wilson et al. 2006; Nguyen et al. 2019) [LIT].</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -11077,10 +11098,32 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="76" t="n"/>
-    </row>
-    <row r="29"/>
-    <row r="30"/>
+      <c r="A28" s="76" t="inlineStr">
+        <is>
+          <t>ferrousGrade_assumption</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>HMS1 equivalent</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>[ASSUMED]</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Assumed grade for FERROUS_METAL(2): HMS1 (Heavy Melting Scrap Grade 1, ≥6mm, clean of non-metallics). Dominant traded grade in Vietnamese industrial scrap markets. See futurenotes.txt [9] for full grading discussion. Price reference: ~280–320 USD/t HCMC 2022–2023 (VASMA, [GREY]).</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Graedel et al. 2011; Daigo et al. 2017; VASMA [GREY] [ASSUMED]</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:E1"/>

</xml_diff>